<commit_message>
Move district dashboards into Districts/, add districts.csv with dashboard links, list all 14 Koshi districts in the Kobo form
</commit_message>
<xml_diff>
--- a/MNH_QI_Tool_XLSFor.xlsx
+++ b/MNH_QI_Tool_XLSFor.xlsx
@@ -10559,7 +10559,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D17"/>
+  <dimension ref="A1:D25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="22" customWidth="1" style="60" min="1" max="2"/>
@@ -10794,17 +10794,17 @@
       </c>
       <c r="B11" s="30" t="inlineStr">
         <is>
-          <t>panchthar</t>
+          <t>bhojpur</t>
         </is>
       </c>
       <c r="C11" s="30" t="inlineStr">
         <is>
-          <t>Panchthar</t>
+          <t>Bhojpur</t>
         </is>
       </c>
       <c r="D11" s="30" t="inlineStr">
         <is>
-          <t>पाँचथर</t>
+          <t>भोजपुर</t>
         </is>
       </c>
     </row>
@@ -10816,17 +10816,17 @@
       </c>
       <c r="B12" s="30" t="inlineStr">
         <is>
-          <t>sankhuwasabha</t>
+          <t>dhankuta</t>
         </is>
       </c>
       <c r="C12" s="30" t="inlineStr">
         <is>
-          <t>Sankhuwasabha</t>
+          <t>Dhankuta</t>
         </is>
       </c>
       <c r="D12" s="30" t="inlineStr">
         <is>
-          <t>संखुवासभा</t>
+          <t>धनकुटा</t>
         </is>
       </c>
     </row>
@@ -10838,17 +10838,17 @@
       </c>
       <c r="B13" s="30" t="inlineStr">
         <is>
-          <t>terhathum</t>
+          <t>ilam</t>
         </is>
       </c>
       <c r="C13" s="30" t="inlineStr">
         <is>
-          <t>Terhathum</t>
+          <t>Ilam</t>
         </is>
       </c>
       <c r="D13" s="30" t="inlineStr">
         <is>
-          <t>तेह्रथुम</t>
+          <t>इलाम</t>
         </is>
       </c>
     </row>
@@ -10860,17 +10860,17 @@
       </c>
       <c r="B14" s="30" t="inlineStr">
         <is>
-          <t>morang</t>
+          <t>jhapa</t>
         </is>
       </c>
       <c r="C14" s="30" t="inlineStr">
         <is>
-          <t>Morang</t>
+          <t>Jhapa</t>
         </is>
       </c>
       <c r="D14" s="30" t="inlineStr">
         <is>
-          <t>मोरङ</t>
+          <t>झापा</t>
         </is>
       </c>
     </row>
@@ -10882,17 +10882,17 @@
       </c>
       <c r="B15" s="30" t="inlineStr">
         <is>
-          <t>sunsari</t>
+          <t>khotang</t>
         </is>
       </c>
       <c r="C15" s="30" t="inlineStr">
         <is>
-          <t>Sunsari</t>
+          <t>Khotang</t>
         </is>
       </c>
       <c r="D15" s="30" t="inlineStr">
         <is>
-          <t>सुनसरी</t>
+          <t>खोटाङ</t>
         </is>
       </c>
     </row>
@@ -10904,17 +10904,17 @@
       </c>
       <c r="B16" s="30" t="inlineStr">
         <is>
-          <t>bhojpur</t>
+          <t>morang</t>
         </is>
       </c>
       <c r="C16" s="30" t="inlineStr">
         <is>
-          <t>Bhojpur</t>
+          <t>Morang</t>
         </is>
       </c>
       <c r="D16" s="30" t="inlineStr">
         <is>
-          <t>भोजपुर</t>
+          <t>मोरङ</t>
         </is>
       </c>
     </row>
@@ -10926,15 +10926,191 @@
       </c>
       <c r="B17" s="30" t="inlineStr">
         <is>
+          <t>okhaldhunga</t>
+        </is>
+      </c>
+      <c r="C17" s="30" t="inlineStr">
+        <is>
+          <t>Okhaldhunga</t>
+        </is>
+      </c>
+      <c r="D17" s="30" t="inlineStr">
+        <is>
+          <t>ओखलढुङ्गा</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="30" t="inlineStr">
+        <is>
+          <t>district</t>
+        </is>
+      </c>
+      <c r="B18" s="30" t="inlineStr">
+        <is>
+          <t>panchthar</t>
+        </is>
+      </c>
+      <c r="C18" s="30" t="inlineStr">
+        <is>
+          <t>Panchthar</t>
+        </is>
+      </c>
+      <c r="D18" s="30" t="inlineStr">
+        <is>
+          <t>पाँचथर</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="30" t="inlineStr">
+        <is>
+          <t>district</t>
+        </is>
+      </c>
+      <c r="B19" s="30" t="inlineStr">
+        <is>
+          <t>sankhuwasabha</t>
+        </is>
+      </c>
+      <c r="C19" s="30" t="inlineStr">
+        <is>
+          <t>Sankhuwasabha</t>
+        </is>
+      </c>
+      <c r="D19" s="30" t="inlineStr">
+        <is>
+          <t>संखुवासभा</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="30" t="inlineStr">
+        <is>
+          <t>district</t>
+        </is>
+      </c>
+      <c r="B20" s="30" t="inlineStr">
+        <is>
+          <t>solukhumbu</t>
+        </is>
+      </c>
+      <c r="C20" s="30" t="inlineStr">
+        <is>
+          <t>Solukhumbu</t>
+        </is>
+      </c>
+      <c r="D20" s="30" t="inlineStr">
+        <is>
+          <t>सोलुखुम्बु</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="30" t="inlineStr">
+        <is>
+          <t>district</t>
+        </is>
+      </c>
+      <c r="B21" s="30" t="inlineStr">
+        <is>
+          <t>sunsari</t>
+        </is>
+      </c>
+      <c r="C21" s="30" t="inlineStr">
+        <is>
+          <t>Sunsari</t>
+        </is>
+      </c>
+      <c r="D21" s="30" t="inlineStr">
+        <is>
+          <t>सुनसरी</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="30" t="inlineStr">
+        <is>
+          <t>district</t>
+        </is>
+      </c>
+      <c r="B22" s="30" t="inlineStr">
+        <is>
+          <t>taplejung</t>
+        </is>
+      </c>
+      <c r="C22" s="30" t="inlineStr">
+        <is>
+          <t>Taplejung</t>
+        </is>
+      </c>
+      <c r="D22" s="30" t="inlineStr">
+        <is>
+          <t>ताप्लेजुङ</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="30" t="inlineStr">
+        <is>
+          <t>district</t>
+        </is>
+      </c>
+      <c r="B23" s="30" t="inlineStr">
+        <is>
+          <t>terhathum</t>
+        </is>
+      </c>
+      <c r="C23" s="30" t="inlineStr">
+        <is>
+          <t>Terhathum</t>
+        </is>
+      </c>
+      <c r="D23" s="30" t="inlineStr">
+        <is>
+          <t>तेह्रथुम</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="30" t="inlineStr">
+        <is>
+          <t>district</t>
+        </is>
+      </c>
+      <c r="B24" s="30" t="inlineStr">
+        <is>
+          <t>udayapur</t>
+        </is>
+      </c>
+      <c r="C24" s="30" t="inlineStr">
+        <is>
+          <t>Udayapur</t>
+        </is>
+      </c>
+      <c r="D24" s="30" t="inlineStr">
+        <is>
+          <t>उदयपुर</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="30" t="inlineStr">
+        <is>
+          <t>district</t>
+        </is>
+      </c>
+      <c r="B25" s="30" t="inlineStr">
+        <is>
           <t>other</t>
         </is>
       </c>
-      <c r="C17" s="30" t="inlineStr">
+      <c r="C25" s="30" t="inlineStr">
         <is>
           <t>Other</t>
         </is>
       </c>
-      <c r="D17" s="30" t="inlineStr">
+      <c r="D25" s="30" t="inlineStr">
         <is>
           <t>अन्य</t>
         </is>
@@ -11007,7 +11183,7 @@
       </c>
       <c r="C2" s="59" t="inlineStr">
         <is>
-          <t>2026.10.06</t>
+          <t>2026.10.06.2</t>
         </is>
       </c>
       <c r="D2" s="59" t="inlineStr">

</xml_diff>